<commit_message>
checkpoint manager for accelerated spinup
</commit_message>
<xml_diff>
--- a/CryoGrid/CryoGridCommunity_results/templates/restart_broken/TILE_LOOP_INIT.xlsx
+++ b/CryoGrid/CryoGridCommunity_results/templates/restart_broken/TILE_LOOP_INIT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Utilisateurs\pozsgayv\Documents\CryoGrid_VP_Workflow\CryoGrid\CryoGridCommunity_results\templates\restart_broken\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D346C33A-068E-42AB-ABB3-C6107042281B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F862298-8CEA-4862-9FDD-F8CBF3EC9436}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="215">
   <si>
     <t>-------------------</t>
   </si>
@@ -667,6 +667,18 @@
   </si>
   <si>
     <t>interval of output files [years]</t>
+  </si>
+  <si>
+    <t>rainfall fraction assumed in sumulations (rainfall from the forcing data file is multiplied by this parameter)</t>
+  </si>
+  <si>
+    <t>snowfall fraction assumed in sumulations (rainfall from the forcing data file is multiplied by this parameter)</t>
+  </si>
+  <si>
+    <t>heat flux at the lower boundary [W/m2] - positive values correspond to energy gain</t>
+  </si>
+  <si>
+    <t>height above ground surface where air temperature from forcing data is applied</t>
   </si>
 </sst>
 </file>
@@ -734,7 +746,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
@@ -746,9 +758,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="11" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1085,142 +1094,142 @@
   <dimension ref="A1:J235"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.81640625" defaultRowHeight="14.5" outlineLevelRow="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.54296875" style="9" customWidth="1"/>
-    <col min="2" max="2" width="19.54296875" style="9" customWidth="1"/>
-    <col min="3" max="3" width="18.54296875" style="9" customWidth="1"/>
-    <col min="4" max="4" width="16.81640625" style="9" customWidth="1"/>
-    <col min="5" max="5" width="16.453125" style="9" customWidth="1"/>
-    <col min="6" max="6" width="30.54296875" style="9" customWidth="1"/>
-    <col min="7" max="7" width="13.453125" style="9" customWidth="1"/>
-    <col min="8" max="8" width="30.08984375" style="9" customWidth="1"/>
-    <col min="9" max="9" width="21.54296875" style="9" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="42.26953125" style="9" customWidth="1"/>
-    <col min="11" max="11" width="9.7265625" style="9" customWidth="1"/>
-    <col min="12" max="12" width="12.1796875" style="9" customWidth="1"/>
-    <col min="13" max="16384" width="8.81640625" style="9"/>
+    <col min="1" max="1" width="23.54296875" style="8" customWidth="1"/>
+    <col min="2" max="2" width="19.54296875" style="8" customWidth="1"/>
+    <col min="3" max="3" width="18.54296875" style="8" customWidth="1"/>
+    <col min="4" max="4" width="16.81640625" style="8" customWidth="1"/>
+    <col min="5" max="5" width="16.453125" style="8" customWidth="1"/>
+    <col min="6" max="6" width="30.54296875" style="8" customWidth="1"/>
+    <col min="7" max="7" width="13.453125" style="8" customWidth="1"/>
+    <col min="8" max="8" width="30.08984375" style="8" customWidth="1"/>
+    <col min="9" max="9" width="21.54296875" style="8" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="42.26953125" style="8" customWidth="1"/>
+    <col min="11" max="11" width="9.7265625" style="8" customWidth="1"/>
+    <col min="12" max="12" width="12.1796875" style="8" customWidth="1"/>
+    <col min="13" max="16384" width="8.81640625" style="8"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" s="9" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="9" t="s">
+      <c r="A2" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="8" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="8" t="s">
         <v>173</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="8" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="8" t="s">
         <v>203</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="D6" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="G6" s="10"/>
+      <c r="G6" s="9"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="9">
-        <v>1</v>
-      </c>
-      <c r="D7" s="9" t="s">
+      <c r="C7" s="8">
+        <v>1</v>
+      </c>
+      <c r="D7" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="G7" s="10"/>
+      <c r="G7" s="9"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="8" t="s">
         <v>174</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="9">
-        <v>1</v>
-      </c>
-      <c r="D8" s="9" t="s">
+      <c r="C8" s="8">
+        <v>1</v>
+      </c>
+      <c r="D8" s="8" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="8" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A12" s="9" t="s">
+      <c r="A12" s="8" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A13" s="9" t="s">
+      <c r="A13" s="8" t="s">
         <v>163</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="8" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="8" t="s">
         <v>164</v>
       </c>
-      <c r="B14" s="9">
+      <c r="B14" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A15" s="9" t="s">
+      <c r="A15" s="8" t="s">
         <v>141</v>
       </c>
       <c r="B15" s="2"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A16" s="9" t="s">
+      <c r="A16" s="8" t="s">
         <v>142</v>
       </c>
       <c r="B16" s="2"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A17" s="9" t="s">
+      <c r="A17" s="8" t="s">
         <v>143</v>
       </c>
       <c r="B17" s="2"/>
@@ -1229,35 +1238,35 @@
       <c r="A18" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="B18" s="11"/>
+      <c r="B18" s="10"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="B19" s="11"/>
+      <c r="B19" s="10"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="B20" s="12"/>
+      <c r="B20" s="11"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A21" s="9" t="s">
+      <c r="A21" s="8" t="s">
         <v>144</v>
       </c>
       <c r="C21" s="3"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A22" s="9" t="s">
+      <c r="A22" s="8" t="s">
         <v>181</v>
       </c>
       <c r="C22" s="3"/>
       <c r="D22" s="1"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A23" s="9" t="s">
+      <c r="A23" s="8" t="s">
         <v>6</v>
       </c>
       <c r="D23" s="1"/>
@@ -1269,40 +1278,40 @@
       <c r="D25" s="1"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A26" s="9" t="s">
+      <c r="A26" s="8" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="9" t="s">
+      <c r="A27" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B27" s="9" t="s">
+      <c r="B27" s="8" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="9" t="s">
+      <c r="A28" s="8" t="s">
         <v>203</v>
       </c>
-      <c r="B28" s="9">
+      <c r="B28" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35"/>
     <row r="30" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="9" t="s">
+      <c r="A30" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B30" s="9" t="s">
+      <c r="B30" s="8" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="31" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="9" t="s">
+      <c r="A31" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="B31" s="9">
+      <c r="B31" s="8">
         <v>100</v>
       </c>
       <c r="C31" s="4" t="s">
@@ -1310,95 +1319,95 @@
       </c>
     </row>
     <row r="32" spans="1:4" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="9" t="s">
+      <c r="A32" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B32" s="13" t="s">
+      <c r="B32" s="12" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="33" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="9" t="s">
+      <c r="A33" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B33" s="9">
+      <c r="B33" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="9" t="s">
+      <c r="A34" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B34" s="9" t="s">
+      <c r="B34" s="8" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="35" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="9" t="s">
+      <c r="A35" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B35" s="9">
+      <c r="B35" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="9" t="s">
+      <c r="A36" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B36" s="9" t="s">
+      <c r="B36" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C36" s="9" t="s">
+      <c r="C36" s="8" t="s">
         <v>197</v>
       </c>
-      <c r="D36" s="9" t="s">
+      <c r="D36" s="8" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="37" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="9" t="s">
+      <c r="A37" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B37" s="9" t="s">
+      <c r="B37" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C37" s="9">
-        <v>1</v>
-      </c>
-      <c r="D37" s="9" t="s">
+      <c r="C37" s="8">
+        <v>1</v>
+      </c>
+      <c r="D37" s="8" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="38" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="9" t="s">
+      <c r="A38" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B38" s="9" t="s">
+      <c r="B38" s="8" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="39" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="9" t="s">
+      <c r="A39" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="B39" s="9">
+      <c r="B39" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="9" t="s">
+      <c r="A40" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="B40" s="9" t="s">
+      <c r="B40" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C40" s="9" t="s">
+      <c r="C40" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="D40" s="9" t="s">
+      <c r="D40" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="E40" s="9" t="s">
+      <c r="E40" s="8" t="s">
         <v>24</v>
       </c>
       <c r="F40" s="4" t="s">
@@ -1406,27 +1415,27 @@
       </c>
     </row>
     <row r="41" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="9" t="s">
+      <c r="A41" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B41" s="9" t="s">
+      <c r="B41" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C41" s="9">
-        <v>1</v>
-      </c>
-      <c r="D41" s="9">
-        <v>1</v>
-      </c>
-      <c r="E41" s="9" t="s">
+      <c r="C41" s="8">
+        <v>1</v>
+      </c>
+      <c r="D41" s="8">
+        <v>1</v>
+      </c>
+      <c r="E41" s="8" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="42" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="9" t="s">
+      <c r="A42" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B42" s="9" t="s">
+      <c r="B42" s="8" t="s">
         <v>27</v>
       </c>
       <c r="C42" s="4" t="s">
@@ -1434,24 +1443,24 @@
       </c>
     </row>
     <row r="43" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="9" t="s">
+      <c r="A43" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="B43" s="9">
+      <c r="B43" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="44" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="9" t="s">
+      <c r="A44" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="B44" s="9" t="s">
+      <c r="B44" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C44" s="9" t="s">
+      <c r="C44" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="D44" s="9" t="s">
+      <c r="D44" s="8" t="s">
         <v>24</v>
       </c>
       <c r="E44" s="4" t="s">
@@ -1459,21 +1468,21 @@
       </c>
     </row>
     <row r="45" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="9" t="s">
+      <c r="A45" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="B45" s="9" t="s">
+      <c r="B45" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C45" s="9">
-        <v>1</v>
-      </c>
-      <c r="D45" s="9" t="s">
+      <c r="C45" s="8">
+        <v>1</v>
+      </c>
+      <c r="D45" s="8" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="46" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="9" t="s">
+      <c r="A46" s="8" t="s">
         <v>168</v>
       </c>
       <c r="C46" s="4" t="s">
@@ -1481,15 +1490,15 @@
       </c>
     </row>
     <row r="47" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="9" t="s">
+      <c r="A47" s="8" t="s">
         <v>169</v>
       </c>
     </row>
     <row r="48" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="9" t="s">
+      <c r="A48" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="B48" s="9">
+      <c r="B48" s="8">
         <v>-2</v>
       </c>
       <c r="C48" s="4" t="s">
@@ -1497,10 +1506,10 @@
       </c>
     </row>
     <row r="49" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="9" t="s">
+      <c r="A49" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="B49" s="9">
+      <c r="B49" s="8">
         <v>0.5</v>
       </c>
       <c r="C49" s="4" t="s">
@@ -1508,7 +1517,7 @@
       </c>
     </row>
     <row r="50" spans="1:6" outlineLevel="1" x14ac:dyDescent="0.35">
-      <c r="A50" s="9" t="s">
+      <c r="A50" s="8" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1517,214 +1526,223 @@
       <c r="D52" s="1"/>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A53" s="9" t="s">
+      <c r="A53" s="8" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A54" s="10" t="s">
+      <c r="A54" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="B54" s="10" t="s">
+      <c r="B54" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="C54" s="10"/>
-      <c r="D54" s="10"/>
-      <c r="E54" s="10"/>
-      <c r="F54" s="10"/>
+      <c r="C54" s="9"/>
+      <c r="D54" s="9"/>
+      <c r="E54" s="9"/>
+      <c r="F54" s="9"/>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A55" s="14" t="s">
+      <c r="A55" s="13" t="s">
         <v>161</v>
       </c>
-      <c r="B55" s="10">
-        <v>1</v>
-      </c>
-      <c r="C55" s="10"/>
-      <c r="D55" s="10"/>
-      <c r="E55" s="10"/>
-      <c r="F55" s="10"/>
+      <c r="B55" s="9">
+        <v>1</v>
+      </c>
+      <c r="C55" s="9"/>
+      <c r="D55" s="9"/>
+      <c r="E55" s="9"/>
+      <c r="F55" s="9"/>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" s="6" t="s">
         <v>32</v>
       </c>
       <c r="B56" s="6"/>
-      <c r="C56" s="10"/>
-      <c r="D56" s="10"/>
-      <c r="E56" s="10"/>
-      <c r="F56" s="10"/>
+      <c r="C56" s="9"/>
+      <c r="D56" s="9"/>
+      <c r="E56" s="9"/>
+      <c r="F56" s="9"/>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A57" s="10" t="s">
+      <c r="A57" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="B57" s="10"/>
-      <c r="C57" s="10"/>
-      <c r="D57" s="10"/>
-      <c r="E57" s="10"/>
-      <c r="F57" s="10"/>
+      <c r="B57" s="9"/>
+      <c r="C57" s="9"/>
+      <c r="D57" s="9"/>
+      <c r="E57" s="9"/>
+      <c r="F57" s="9"/>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A58" s="10" t="s">
+      <c r="A58" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="B58" s="10"/>
+      <c r="B58" s="9"/>
       <c r="C58" s="6"/>
       <c r="D58" s="6"/>
       <c r="E58" s="6"/>
-      <c r="F58" s="10"/>
+      <c r="F58" s="9"/>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A59" s="10" t="s">
+      <c r="A59" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B59" s="10"/>
+      <c r="B59" s="9"/>
       <c r="C59" s="6"/>
       <c r="D59" s="6"/>
       <c r="E59" s="6"/>
-      <c r="F59" s="10"/>
+      <c r="F59" s="9"/>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A60" s="10" t="s">
+      <c r="A60" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B60" s="10">
-        <v>1</v>
-      </c>
-      <c r="C60" s="10"/>
-      <c r="D60" s="10"/>
-      <c r="E60" s="10"/>
-      <c r="F60" s="10"/>
+      <c r="B60">
+        <v>1</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="D60" s="9"/>
+      <c r="E60" s="9"/>
+      <c r="F60" s="9"/>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B61" s="7">
-        <v>1</v>
-      </c>
-      <c r="C61" s="10"/>
-      <c r="D61" s="10"/>
-      <c r="E61" s="10"/>
-      <c r="F61" s="10"/>
+      <c r="B61">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="D61" s="9"/>
+      <c r="E61" s="9"/>
+      <c r="F61" s="9"/>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A62" s="10" t="s">
+      <c r="A62" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="B62" s="10">
+      <c r="B62">
+        <v>0.05</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="D62" s="9"/>
+      <c r="E62" s="9"/>
+      <c r="F62" s="9"/>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A63" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B63">
+        <v>2</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A64" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="B64" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C64" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="D64" s="8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A65" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="B65" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C65" s="8">
+        <v>1</v>
+      </c>
+      <c r="D65" s="8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A66" s="8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A68" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="B68" s="8" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A69" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="B69" s="8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A70" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="B70" s="8">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A71" s="8" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A74" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="C62" s="10"/>
-      <c r="D62" s="10"/>
-      <c r="E62" s="10"/>
-      <c r="F62" s="10"/>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A63" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="B63" s="9">
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A75" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B75" s="8" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A64" s="9" t="s">
-        <v>120</v>
-      </c>
-      <c r="B64" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="C64" s="9" t="s">
-        <v>160</v>
-      </c>
-      <c r="D64" s="9" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A65" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="B65" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="C65" s="9">
-        <v>1</v>
-      </c>
-      <c r="D65" s="9" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A66" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A68" s="9" t="s">
-        <v>165</v>
-      </c>
-      <c r="B68" s="9" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A69" s="9" t="s">
-        <v>160</v>
-      </c>
-      <c r="B69" s="9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A70" s="9" t="s">
-        <v>166</v>
-      </c>
-      <c r="B70" s="9">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A71" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A74" s="9" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A75" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="B75" s="9" t="s">
-        <v>2</v>
-      </c>
-    </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A76" s="9" t="s">
+      <c r="A76" s="8" t="s">
         <v>200</v>
       </c>
-      <c r="B76" s="9">
+      <c r="B76" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C77" s="9" t="s">
+      <c r="C77" s="8" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A78" s="9" t="s">
+      <c r="A78" s="8" t="s">
         <v>201</v>
       </c>
-      <c r="B78" s="9">
+      <c r="B78" s="8">
         <v>5</v>
       </c>
-      <c r="C78" s="9">
+      <c r="C78" s="8">
         <v>5</v>
       </c>
       <c r="D78" s="4" t="s">
@@ -1732,28 +1750,28 @@
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A79" s="9" t="s">
+      <c r="A79" s="8" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A82" s="9" t="s">
+      <c r="A82" s="8" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A83" s="9" t="s">
+      <c r="A83" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="B83" s="9" t="s">
+      <c r="B83" s="8" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A84" s="9" t="s">
+      <c r="A84" s="8" t="s">
         <v>197</v>
       </c>
-      <c r="B84" s="9">
+      <c r="B84" s="8">
         <v>1</v>
       </c>
     </row>
@@ -1815,146 +1833,146 @@
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A94" s="9" t="s">
+      <c r="A94" s="8" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A95" s="9" t="s">
+      <c r="A95" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="B95" s="9" t="s">
+      <c r="B95" s="8" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A96" s="9" t="s">
+      <c r="A96" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="B96" s="9">
+      <c r="B96" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A98" s="9" t="s">
+      <c r="A98" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="B98" s="9" t="s">
+      <c r="B98" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="C98" s="9" t="s">
+      <c r="C98" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="D98" s="9" t="s">
+      <c r="D98" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="E98" s="9" t="s">
+      <c r="E98" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="F98" s="9" t="s">
+      <c r="F98" s="8" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="C99" s="9">
+      <c r="C99" s="8">
         <v>0</v>
       </c>
-      <c r="D99" s="15">
+      <c r="D99" s="14">
         <v>0.05</v>
       </c>
-      <c r="E99" s="9">
+      <c r="E99" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="C100" s="9">
+      <c r="C100" s="8">
         <v>0.5</v>
       </c>
-      <c r="D100" s="15">
+      <c r="D100" s="14">
         <v>0.05</v>
       </c>
-      <c r="E100" s="9">
+      <c r="E100" s="8">
         <v>3</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="C101" s="9">
+      <c r="C101" s="8">
         <v>3</v>
       </c>
-      <c r="D101" s="15">
+      <c r="D101" s="14">
         <v>0.1</v>
       </c>
-      <c r="E101" s="9">
+      <c r="E101" s="8">
         <v>10</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="C102" s="9">
+      <c r="C102" s="8">
         <v>10</v>
       </c>
-      <c r="D102" s="9">
-        <v>1</v>
-      </c>
-      <c r="E102" s="9">
+      <c r="D102" s="8">
+        <v>1</v>
+      </c>
+      <c r="E102" s="8">
         <v>50</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="C103" s="9">
+      <c r="C103" s="8">
         <v>50</v>
       </c>
-      <c r="D103" s="15">
+      <c r="D103" s="14">
         <v>5</v>
       </c>
-      <c r="E103" s="9">
+      <c r="E103" s="8">
         <v>100</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="B104" s="9" t="s">
+      <c r="B104" s="8" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A105" s="9" t="s">
+      <c r="A105" s="8" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A108" s="9" t="s">
+      <c r="A108" s="8" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A109" s="9" t="s">
+      <c r="A109" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="B109" s="9" t="s">
+      <c r="B109" s="8" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A110" s="9" t="s">
+      <c r="A110" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B110" s="9">
+      <c r="B110" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A112" s="9" t="s">
+      <c r="A112" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="B112" s="9" t="s">
+      <c r="B112" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="C112" s="9" t="s">
+      <c r="C112" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="D112" s="9" t="s">
+      <c r="D112" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="E112" s="9" t="s">
+      <c r="E112" s="8" t="s">
         <v>24</v>
       </c>
       <c r="F112" s="4" t="s">
@@ -1962,24 +1980,24 @@
       </c>
     </row>
     <row r="113" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B113" s="9">
+      <c r="B113" s="8">
         <v>0</v>
       </c>
-      <c r="C113" s="9" t="s">
+      <c r="C113" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="D113" s="9">
+      <c r="D113" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="114" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B114" s="9">
+      <c r="B114" s="8">
         <v>5</v>
       </c>
-      <c r="C114" s="9" t="s">
+      <c r="C114" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="D114" s="9">
+      <c r="D114" s="8">
         <v>1</v>
       </c>
       <c r="F114" s="4" t="s">
@@ -1987,15 +2005,15 @@
       </c>
     </row>
     <row r="115" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B115" s="9" t="s">
+      <c r="B115" s="8" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="116" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A116" s="9" t="s">
+      <c r="A116" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="B116" s="9" t="s">
+      <c r="B116" s="8" t="s">
         <v>145</v>
       </c>
       <c r="D116" s="4" t="s">
@@ -2003,21 +2021,21 @@
       </c>
     </row>
     <row r="117" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A117" s="9" t="s">
+      <c r="A117" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="B117" s="9">
+      <c r="B117" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="118" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A118" s="9" t="s">
+      <c r="A118" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="B118" s="9" t="s">
+      <c r="B118" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C118" s="9" t="s">
+      <c r="C118" s="8" t="s">
         <v>24</v>
       </c>
       <c r="D118" s="4" t="s">
@@ -2025,74 +2043,74 @@
       </c>
     </row>
     <row r="119" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A119" s="9" t="s">
+      <c r="A119" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="B119" s="9" t="s">
+      <c r="B119" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="C119" s="9" t="s">
+      <c r="C119" s="8" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="120" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A120" s="9" t="s">
+      <c r="A120" s="8" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="123" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A123" s="9" t="s">
+      <c r="A123" s="8" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="124" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A124" s="9" t="s">
+      <c r="A124" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="B124" s="9" t="s">
+      <c r="B124" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D124" s="16" t="s">
+      <c r="D124" s="15" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="125" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A125" s="9" t="s">
+      <c r="A125" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B125" s="9">
-        <v>1</v>
-      </c>
-      <c r="D125" s="16" t="s">
+      <c r="B125" s="8">
+        <v>1</v>
+      </c>
+      <c r="D125" s="15" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="127" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A127" s="9" t="s">
+      <c r="A127" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="B127" s="9" t="s">
+      <c r="B127" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="C127" s="9" t="s">
+      <c r="C127" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="D127" s="9" t="s">
+      <c r="D127" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="E127" s="9" t="s">
+      <c r="E127" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="F127" s="9" t="s">
+      <c r="F127" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="G127" s="9" t="s">
+      <c r="G127" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="H127" s="9" t="s">
+      <c r="H127" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="I127" s="9" t="s">
+      <c r="I127" s="8" t="s">
         <v>24</v>
       </c>
       <c r="J127" s="4" t="s">
@@ -2100,143 +2118,143 @@
       </c>
     </row>
     <row r="128" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="B128" s="9">
+      <c r="B128" s="8">
         <v>0</v>
       </c>
-      <c r="C128" s="9">
+      <c r="C128" s="8">
         <v>0.4</v>
       </c>
-      <c r="D128" s="9">
+      <c r="D128" s="8">
         <v>0.6</v>
       </c>
-      <c r="E128" s="9">
+      <c r="E128" s="8">
         <v>0</v>
       </c>
-      <c r="F128" s="9">
+      <c r="F128" s="8">
         <v>2</v>
       </c>
-      <c r="G128" s="9">
+      <c r="G128" s="8">
         <v>0.2</v>
       </c>
-      <c r="H128" s="8">
+      <c r="H128" s="7">
         <v>9.9999999999999995E-7</v>
       </c>
     </row>
     <row r="129" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B129" s="9">
+      <c r="B129" s="8">
         <v>0.1</v>
       </c>
-      <c r="C129" s="9">
+      <c r="C129" s="8">
         <v>0.4</v>
       </c>
-      <c r="D129" s="9">
+      <c r="D129" s="8">
         <v>0.6</v>
       </c>
-      <c r="E129" s="9">
+      <c r="E129" s="8">
         <v>0</v>
       </c>
-      <c r="F129" s="9">
+      <c r="F129" s="8">
         <v>2</v>
       </c>
-      <c r="G129" s="9">
+      <c r="G129" s="8">
         <v>0.2</v>
       </c>
-      <c r="H129" s="8">
+      <c r="H129" s="7">
         <v>9.9999999999999995E-7</v>
       </c>
     </row>
     <row r="130" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B130" s="9">
+      <c r="B130" s="8">
         <v>5</v>
       </c>
-      <c r="C130" s="9">
+      <c r="C130" s="8">
         <v>0.03</v>
       </c>
-      <c r="D130" s="9">
+      <c r="D130" s="8">
         <v>0.97</v>
       </c>
-      <c r="E130" s="9">
+      <c r="E130" s="8">
         <v>0</v>
       </c>
-      <c r="F130" s="9">
-        <v>1</v>
-      </c>
-      <c r="G130" s="9">
+      <c r="F130" s="8">
+        <v>1</v>
+      </c>
+      <c r="G130" s="8">
         <v>0.03</v>
       </c>
-      <c r="H130" s="8">
+      <c r="H130" s="7">
         <v>9.9999999999999995E-7</v>
       </c>
     </row>
     <row r="131" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="B131" s="9" t="s">
+      <c r="B131" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="G131" s="16" t="s">
+      <c r="G131" s="15" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="132" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A132" s="9" t="s">
+      <c r="A132" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="G132" s="16" t="s">
+      <c r="G132" s="15" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="133" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="G133" s="16" t="s">
+      <c r="G133" s="15" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="134" spans="1:8" s="10" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="134" spans="1:8" s="9" customFormat="1" x14ac:dyDescent="0.35"/>
     <row r="135" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A135" s="10" t="s">
+      <c r="A135" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B135" s="10"/>
-      <c r="C135" s="10"/>
+      <c r="B135" s="9"/>
+      <c r="C135" s="9"/>
     </row>
     <row r="136" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A136" s="10" t="s">
+      <c r="A136" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="B136" s="10" t="s">
+      <c r="B136" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="C136" s="10"/>
+      <c r="C136" s="9"/>
     </row>
     <row r="137" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A137" s="10" t="s">
+      <c r="A137" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="B137" s="10">
-        <v>1</v>
-      </c>
-      <c r="C137" s="10"/>
+      <c r="B137" s="9">
+        <v>1</v>
+      </c>
+      <c r="C137" s="9"/>
     </row>
     <row r="138" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A138" s="10"/>
-      <c r="B138" s="10"/>
-      <c r="C138" s="10"/>
+      <c r="A138" s="9"/>
+      <c r="B138" s="9"/>
+      <c r="C138" s="9"/>
     </row>
     <row r="139" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A139" s="10" t="s">
+      <c r="A139" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="B139" s="10" t="s">
+      <c r="B139" s="9" t="s">
         <v>52</v>
       </c>
       <c r="C139" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D139" s="9" t="s">
+      <c r="D139" s="8" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="140" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A140" s="10"/>
-      <c r="B140" s="10">
+      <c r="A140" s="9"/>
+      <c r="B140" s="9">
         <v>0</v>
       </c>
       <c r="C140" s="6">
@@ -2244,70 +2262,70 @@
       </c>
     </row>
     <row r="141" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A141" s="10"/>
+      <c r="A141" s="9"/>
       <c r="B141" s="6">
         <v>100</v>
       </c>
       <c r="C141" s="6">
         <v>-2</v>
       </c>
-      <c r="D141" s="9" t="s">
+      <c r="D141" s="8" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="142" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A142" s="10"/>
-      <c r="B142" s="10" t="s">
+      <c r="A142" s="9"/>
+      <c r="B142" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="C142" s="17"/>
+      <c r="C142" s="16"/>
     </row>
     <row r="143" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A143" s="10" t="s">
+      <c r="A143" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B143" s="10"/>
-      <c r="C143" s="10"/>
+      <c r="B143" s="9"/>
+      <c r="C143" s="9"/>
     </row>
     <row r="144" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A144" s="10"/>
-      <c r="B144" s="10"/>
-      <c r="C144" s="10"/>
+      <c r="A144" s="9"/>
+      <c r="B144" s="9"/>
+      <c r="C144" s="9"/>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A145" s="10"/>
-      <c r="B145" s="10"/>
-      <c r="C145" s="10"/>
+      <c r="A145" s="9"/>
+      <c r="B145" s="9"/>
+      <c r="C145" s="9"/>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A146" s="10" t="s">
+      <c r="A146" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B146" s="10"/>
-      <c r="C146" s="10"/>
+      <c r="B146" s="9"/>
+      <c r="C146" s="9"/>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A147" s="10" t="s">
+      <c r="A147" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="B147" s="10" t="s">
+      <c r="B147" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="C147" s="10"/>
+      <c r="C147" s="9"/>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A148" s="10" t="s">
+      <c r="A148" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="B148" s="10">
-        <v>1</v>
-      </c>
-      <c r="C148" s="10"/>
+      <c r="B148" s="9">
+        <v>1</v>
+      </c>
+      <c r="C148" s="9"/>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A149" s="10"/>
-      <c r="B149" s="10"/>
-      <c r="C149" s="10" t="s">
+      <c r="A149" s="9"/>
+      <c r="B149" s="9"/>
+      <c r="C149" s="9" t="s">
         <v>3</v>
       </c>
     </row>
@@ -2318,7 +2336,7 @@
       <c r="B150" s="6">
         <v>0.25</v>
       </c>
-      <c r="C150" s="10">
+      <c r="C150" s="9">
         <v>0.2</v>
       </c>
       <c r="D150" s="4" t="s">
@@ -2326,13 +2344,13 @@
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A151" s="10" t="s">
+      <c r="A151" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="B151" s="10">
+      <c r="B151" s="9">
         <v>0.99</v>
       </c>
-      <c r="C151" s="10">
+      <c r="C151" s="9">
         <v>0.99</v>
       </c>
       <c r="D151" s="4" t="s">
@@ -2340,13 +2358,13 @@
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A152" s="10" t="s">
+      <c r="A152" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="B152" s="10">
+      <c r="B152" s="9">
         <v>0.27</v>
       </c>
-      <c r="C152" s="10">
+      <c r="C152" s="9">
         <v>0.01</v>
       </c>
       <c r="D152" s="4" t="s">
@@ -2354,13 +2372,13 @@
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A153" s="10" t="s">
+      <c r="A153" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="B153" s="10">
+      <c r="B153" s="9">
         <v>0.1</v>
       </c>
-      <c r="C153" s="10">
+      <c r="C153" s="9">
         <v>0.1</v>
       </c>
       <c r="D153" s="4" t="s">
@@ -2368,13 +2386,13 @@
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A154" s="10" t="s">
+      <c r="A154" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="B154" s="10">
+      <c r="B154" s="9">
         <v>0.1</v>
       </c>
-      <c r="C154" s="10">
+      <c r="C154" s="9">
         <v>0.1</v>
       </c>
       <c r="D154" s="4" t="s">
@@ -2382,13 +2400,13 @@
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A155" s="10" t="s">
+      <c r="A155" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="B155" s="10">
+      <c r="B155" s="9">
         <v>0.5</v>
       </c>
-      <c r="C155" s="10">
+      <c r="C155" s="9">
         <v>0.5</v>
       </c>
       <c r="D155" s="4" t="s">
@@ -2396,13 +2414,13 @@
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A156" s="10" t="s">
+      <c r="A156" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="B156" s="10">
+      <c r="B156" s="9">
         <v>1.0000000000000001E-5</v>
       </c>
-      <c r="C156" s="10">
+      <c r="C156" s="9">
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="D156" s="4" t="s">
@@ -2410,13 +2428,13 @@
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A157" s="10" t="s">
+      <c r="A157" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="B157" s="10" t="s">
+      <c r="B157" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="C157" s="10" t="s">
+      <c r="C157" s="9" t="s">
         <v>77</v>
       </c>
       <c r="D157" s="4" t="s">
@@ -2424,13 +2442,13 @@
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A158" s="9" t="s">
+      <c r="A158" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="B158" s="9">
+      <c r="B158" s="8">
         <v>3600</v>
       </c>
-      <c r="C158" s="9">
+      <c r="C158" s="8">
         <v>3600</v>
       </c>
       <c r="D158" s="4" t="s">
@@ -2438,13 +2456,13 @@
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A159" s="9" t="s">
+      <c r="A159" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="B159" s="9">
+      <c r="B159" s="8">
         <v>50000</v>
       </c>
-      <c r="C159" s="9">
+      <c r="C159" s="8">
         <v>50000</v>
       </c>
       <c r="D159" s="4" t="s">
@@ -2452,13 +2470,13 @@
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A160" s="9" t="s">
+      <c r="A160" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="B160" s="9">
+      <c r="B160" s="8">
         <v>1000</v>
       </c>
-      <c r="C160" s="9">
+      <c r="C160" s="8">
         <v>1000</v>
       </c>
       <c r="D160" s="4" t="s">
@@ -2466,13 +2484,13 @@
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A161" s="9" t="s">
+      <c r="A161" s="8" t="s">
         <v>139</v>
       </c>
-      <c r="B161" s="9">
+      <c r="B161" s="8">
         <v>1000</v>
       </c>
-      <c r="C161" s="9">
+      <c r="C161" s="8">
         <v>1000</v>
       </c>
       <c r="D161" s="4" t="s">
@@ -2480,13 +2498,13 @@
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A162" s="9" t="s">
+      <c r="A162" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="B162" s="9">
+      <c r="B162" s="8">
         <v>-40</v>
       </c>
-      <c r="C162" s="9">
+      <c r="C162" s="8">
         <v>-50</v>
       </c>
       <c r="D162" s="4" t="s">
@@ -2494,13 +2512,13 @@
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A163" s="9" t="s">
+      <c r="A163" s="8" t="s">
         <v>131</v>
       </c>
-      <c r="B163" s="9">
+      <c r="B163" s="8">
         <v>0.05</v>
       </c>
-      <c r="C163" s="9">
+      <c r="C163" s="8">
         <v>0.05</v>
       </c>
       <c r="D163" s="4" t="s">
@@ -2508,13 +2526,13 @@
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A164" s="9" t="s">
+      <c r="A164" s="8" t="s">
         <v>133</v>
       </c>
-      <c r="B164" s="9">
+      <c r="B164" s="8">
         <v>0.97</v>
       </c>
-      <c r="C164" s="9">
+      <c r="C164" s="8">
         <v>0.97</v>
       </c>
       <c r="D164" s="4" t="s">
@@ -2522,13 +2540,13 @@
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A165" s="9" t="s">
+      <c r="A165" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="B165" s="9">
+      <c r="B165" s="8">
         <v>0.03</v>
       </c>
-      <c r="C165" s="9">
+      <c r="C165" s="8">
         <v>0.03</v>
       </c>
       <c r="D165" s="4" t="s">
@@ -2536,44 +2554,44 @@
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A166" s="9" t="s">
+      <c r="A166" s="8" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A169" s="9" t="s">
+      <c r="A169" s="8" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A170" s="9" t="s">
+      <c r="A170" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="B170" s="9" t="s">
+      <c r="B170" s="8" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A171" s="9" t="s">
+      <c r="A171" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="B171" s="9">
+      <c r="B171" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C172" s="9" t="s">
+      <c r="C172" s="8" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A173" s="9" t="s">
+      <c r="A173" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="B173" s="9">
+      <c r="B173" s="8">
         <v>0.25</v>
       </c>
-      <c r="C173" s="9">
+      <c r="C173" s="8">
         <v>0.2</v>
       </c>
       <c r="D173" s="4" t="s">
@@ -2581,13 +2599,13 @@
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A174" s="9" t="s">
+      <c r="A174" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="B174" s="9">
+      <c r="B174" s="8">
         <v>0.99</v>
       </c>
-      <c r="C174" s="9">
+      <c r="C174" s="8">
         <v>0.99</v>
       </c>
       <c r="D174" s="4" t="s">
@@ -2595,13 +2613,13 @@
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A175" s="9" t="s">
+      <c r="A175" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="B175" s="10">
+      <c r="B175" s="9">
         <v>0.27</v>
       </c>
-      <c r="C175" s="9">
+      <c r="C175" s="8">
         <v>0.01</v>
       </c>
       <c r="D175" s="4" t="s">
@@ -2609,13 +2627,13 @@
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A176" s="9" t="s">
+      <c r="A176" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="B176" s="9">
+      <c r="B176" s="8">
         <v>0</v>
       </c>
-      <c r="C176" s="9">
+      <c r="C176" s="8">
         <v>0</v>
       </c>
       <c r="D176" s="4" t="s">
@@ -2623,13 +2641,13 @@
       </c>
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A177" s="9" t="s">
+      <c r="A177" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="B177" s="9" t="s">
+      <c r="B177" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="C177" s="9" t="s">
+      <c r="C177" s="8" t="s">
         <v>77</v>
       </c>
       <c r="D177" s="4" t="s">
@@ -2637,13 +2655,13 @@
       </c>
     </row>
     <row r="178" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A178" s="9" t="s">
+      <c r="A178" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="B178" s="9">
+      <c r="B178" s="8">
         <v>3600</v>
       </c>
-      <c r="C178" s="9">
+      <c r="C178" s="8">
         <v>3600</v>
       </c>
       <c r="D178" s="4" t="s">
@@ -2651,13 +2669,13 @@
       </c>
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A179" s="9" t="s">
+      <c r="A179" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="B179" s="9">
+      <c r="B179" s="8">
         <v>50000</v>
       </c>
-      <c r="C179" s="9">
+      <c r="C179" s="8">
         <v>50000</v>
       </c>
       <c r="D179" s="4" t="s">
@@ -2665,44 +2683,44 @@
       </c>
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A180" s="9" t="s">
+      <c r="A180" s="8" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="183" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A183" s="9" t="s">
+      <c r="A183" s="8" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="184" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A184" s="9" t="s">
+      <c r="A184" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="B184" s="9" t="s">
+      <c r="B184" s="8" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="185" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A185" s="9" t="s">
+      <c r="A185" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="B185" s="9">
+      <c r="B185" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="186" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C186" s="9" t="s">
+      <c r="C186" s="8" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="187" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A187" s="9" t="s">
+      <c r="A187" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="B187" s="9">
+      <c r="B187" s="8">
         <v>0.99</v>
       </c>
-      <c r="C187" s="9">
+      <c r="C187" s="8">
         <v>0.99</v>
       </c>
       <c r="D187" s="4" t="s">
@@ -2710,13 +2728,13 @@
       </c>
     </row>
     <row r="188" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A188" s="9" t="s">
+      <c r="A188" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="B188" s="9">
+      <c r="B188" s="8">
         <v>1E-3</v>
       </c>
-      <c r="C188" s="9">
+      <c r="C188" s="8">
         <v>0.01</v>
       </c>
       <c r="D188" s="4" t="s">
@@ -2724,13 +2742,13 @@
       </c>
     </row>
     <row r="189" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A189" s="9" t="s">
+      <c r="A189" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="B189" s="9">
+      <c r="B189" s="8">
         <v>0.71</v>
       </c>
-      <c r="C189" s="9">
+      <c r="C189" s="8">
         <v>0.71</v>
       </c>
       <c r="D189" s="4" t="s">
@@ -2738,13 +2756,13 @@
       </c>
     </row>
     <row r="190" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A190" s="9" t="s">
+      <c r="A190" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="B190" s="9">
+      <c r="B190" s="8">
         <v>0.21</v>
       </c>
-      <c r="C190" s="9">
+      <c r="C190" s="8">
         <v>0.21</v>
       </c>
       <c r="D190" s="4" t="s">
@@ -2752,7 +2770,7 @@
       </c>
     </row>
     <row r="191" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A191" s="9" t="s">
+      <c r="A191" s="8" t="s">
         <v>88</v>
       </c>
       <c r="D191" s="4" t="s">
@@ -2760,13 +2778,13 @@
       </c>
     </row>
     <row r="192" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A192" s="9" t="s">
+      <c r="A192" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="B192" s="9">
+      <c r="B192" s="8">
         <v>0.05</v>
       </c>
-      <c r="C192" s="9">
+      <c r="C192" s="8">
         <v>0.05</v>
       </c>
       <c r="D192" s="4" t="s">
@@ -2774,13 +2792,13 @@
       </c>
     </row>
     <row r="193" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A193" s="9" t="s">
+      <c r="A193" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="B193" s="9">
+      <c r="B193" s="8">
         <v>1E-4</v>
       </c>
-      <c r="C193" s="9">
+      <c r="C193" s="8">
         <v>1E-4</v>
       </c>
       <c r="D193" s="4" t="s">
@@ -2788,13 +2806,13 @@
       </c>
     </row>
     <row r="194" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A194" s="9" t="s">
+      <c r="A194" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="B194" s="9">
+      <c r="B194" s="8">
         <v>0.01</v>
       </c>
-      <c r="C194" s="9">
+      <c r="C194" s="8">
         <v>0.02</v>
       </c>
       <c r="D194" s="4" t="s">
@@ -2802,13 +2820,13 @@
       </c>
     </row>
     <row r="195" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A195" s="9" t="s">
+      <c r="A195" s="8" t="s">
         <v>194</v>
       </c>
-      <c r="B195" s="9">
+      <c r="B195" s="8">
         <v>0</v>
       </c>
-      <c r="C195" s="9">
+      <c r="C195" s="8">
         <v>0</v>
       </c>
       <c r="D195" s="4" t="s">
@@ -2816,14 +2834,14 @@
       </c>
     </row>
     <row r="196" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A196" s="9" t="s">
+      <c r="A196" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="B196" s="9">
+      <c r="B196" s="8">
         <f>48/3</f>
         <v>16</v>
       </c>
-      <c r="C196" s="9">
+      <c r="C196" s="8">
         <v>48</v>
       </c>
       <c r="D196" s="4" t="s">
@@ -2831,13 +2849,13 @@
       </c>
     </row>
     <row r="197" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A197" s="9" t="s">
+      <c r="A197" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="B197" s="9">
+      <c r="B197" s="8">
         <v>600</v>
       </c>
-      <c r="C197" s="9">
+      <c r="C197" s="8">
         <v>350</v>
       </c>
       <c r="D197" s="4" t="s">
@@ -2845,13 +2863,13 @@
       </c>
     </row>
     <row r="198" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A198" s="9" t="s">
+      <c r="A198" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="B198" s="9">
+      <c r="B198" s="8">
         <v>52</v>
       </c>
-      <c r="C198" s="9">
+      <c r="C198" s="8">
         <v>26</v>
       </c>
       <c r="D198" s="4" t="s">
@@ -2859,10 +2877,10 @@
       </c>
     </row>
     <row r="199" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A199" s="9" t="s">
+      <c r="A199" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="B199" s="9">
+      <c r="B199" s="8">
         <f>0.06/60</f>
         <v>1E-3</v>
       </c>
@@ -2871,13 +2889,13 @@
       </c>
     </row>
     <row r="200" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A200" s="9" t="s">
+      <c r="A200" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="B200" s="9" t="s">
+      <c r="B200" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="C200" s="9" t="s">
+      <c r="C200" s="8" t="s">
         <v>196</v>
       </c>
       <c r="D200" s="4" t="s">
@@ -2885,13 +2903,13 @@
       </c>
     </row>
     <row r="201" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A201" s="9" t="s">
+      <c r="A201" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="B201" s="9">
+      <c r="B201" s="8">
         <v>3600</v>
       </c>
-      <c r="C201" s="9">
+      <c r="C201" s="8">
         <v>3600</v>
       </c>
       <c r="D201" s="4" t="s">
@@ -2899,13 +2917,13 @@
       </c>
     </row>
     <row r="202" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A202" s="9" t="s">
+      <c r="A202" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="B202" s="9">
+      <c r="B202" s="8">
         <v>50000</v>
       </c>
-      <c r="C202" s="9">
+      <c r="C202" s="8">
         <v>50000</v>
       </c>
       <c r="D202" s="4" t="s">
@@ -2913,13 +2931,13 @@
       </c>
     </row>
     <row r="203" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A203" s="9" t="s">
+      <c r="A203" s="8" t="s">
         <v>122</v>
       </c>
       <c r="D203" s="4"/>
     </row>
     <row r="204" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A204" s="9" t="s">
+      <c r="A204" s="8" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2930,23 +2948,23 @@
       <c r="D206" s="4"/>
     </row>
     <row r="207" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A207" s="9" t="s">
+      <c r="A207" s="8" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="208" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A208" s="9" t="s">
+      <c r="A208" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="B208" s="9" t="s">
+      <c r="B208" s="8" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="209" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A209" s="9" t="s">
+      <c r="A209" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="B209" s="9">
+      <c r="B209" s="8">
         <v>1</v>
       </c>
       <c r="D209" s="4" t="s">
@@ -2954,18 +2972,18 @@
       </c>
     </row>
     <row r="210" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C210" s="9" t="s">
+      <c r="C210" s="8" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A211" s="9" t="s">
+      <c r="A211" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="B211" s="9">
+      <c r="B211" s="8">
         <v>0.25</v>
       </c>
-      <c r="C211" s="9">
+      <c r="C211" s="8">
         <v>0.25</v>
       </c>
       <c r="D211" s="4" t="s">
@@ -2973,7 +2991,7 @@
       </c>
     </row>
     <row r="212" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A212" s="9" t="s">
+      <c r="A212" s="8" t="s">
         <v>6</v>
       </c>
     </row>
@@ -2984,39 +3002,39 @@
       <c r="D214" s="4"/>
     </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A215" s="9" t="s">
+      <c r="A215" s="8" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="216" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A216" s="9" t="s">
+      <c r="A216" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="B216" s="9" t="s">
+      <c r="B216" s="8" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="217" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A217" s="9" t="s">
+      <c r="A217" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="B217" s="9">
+      <c r="B217" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="218" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="C218" s="9" t="s">
+      <c r="C218" s="8" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="219" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A219" s="9" t="s">
+      <c r="A219" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="B219" s="9">
+      <c r="B219" s="8">
         <v>20</v>
       </c>
-      <c r="C219" s="9">
+      <c r="C219" s="8">
         <v>10000</v>
       </c>
       <c r="D219" s="4" t="s">
@@ -3024,13 +3042,13 @@
       </c>
     </row>
     <row r="220" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A220" s="9" t="s">
+      <c r="A220" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="B220" s="9">
+      <c r="B220" s="8">
         <v>0</v>
       </c>
-      <c r="C220" s="9">
+      <c r="C220" s="8">
         <v>0</v>
       </c>
       <c r="D220" s="4" t="s">
@@ -3038,13 +3056,13 @@
       </c>
     </row>
     <row r="221" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A221" s="9" t="s">
+      <c r="A221" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="B221" s="9">
+      <c r="B221" s="8">
         <v>0.03</v>
       </c>
-      <c r="C221" s="9">
+      <c r="C221" s="8">
         <v>0.03</v>
       </c>
       <c r="D221" s="4" t="s">
@@ -3052,13 +3070,13 @@
       </c>
     </row>
     <row r="222" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A222" s="9" t="s">
+      <c r="A222" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="B222" s="9">
+      <c r="B222" s="8">
         <v>5</v>
       </c>
-      <c r="C222" s="9">
+      <c r="C222" s="8">
         <v>1</v>
       </c>
       <c r="D222" s="4" t="s">
@@ -3066,13 +3084,13 @@
       </c>
     </row>
     <row r="223" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A223" s="9" t="s">
+      <c r="A223" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="B223" s="9">
-        <v>1</v>
-      </c>
-      <c r="C223" s="9">
+      <c r="B223" s="8">
+        <v>1</v>
+      </c>
+      <c r="C223" s="8">
         <v>1</v>
       </c>
       <c r="D223" s="4" t="s">
@@ -3080,7 +3098,7 @@
       </c>
     </row>
     <row r="224" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A224" s="9" t="s">
+      <c r="A224" s="8" t="s">
         <v>6</v>
       </c>
     </row>
@@ -3091,25 +3109,25 @@
       <c r="D226" s="4"/>
     </row>
     <row r="227" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A227" s="18" t="s">
+      <c r="A227" s="17" t="s">
         <v>148</v>
       </c>
       <c r="D227" s="4"/>
     </row>
     <row r="228" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A228" s="9" t="s">
+      <c r="A228" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="B228" s="9" t="s">
+      <c r="B228" s="8" t="s">
         <v>2</v>
       </c>
       <c r="D228" s="4"/>
     </row>
     <row r="229" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A229" s="9" t="s">
+      <c r="A229" s="8" t="s">
         <v>147</v>
       </c>
-      <c r="B229" s="9">
+      <c r="B229" s="8">
         <v>1</v>
       </c>
       <c r="D229" s="4"/>
@@ -3131,7 +3149,7 @@
       <c r="D231" s="4"/>
     </row>
     <row r="232" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A232" s="9" t="s">
+      <c r="A232" s="8" t="s">
         <v>112</v>
       </c>
       <c r="B232" s="2">
@@ -3140,7 +3158,7 @@
       <c r="D232" s="4"/>
     </row>
     <row r="233" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A233" s="9" t="s">
+      <c r="A233" s="8" t="s">
         <v>150</v>
       </c>
       <c r="B233" s="2">
@@ -3160,7 +3178,7 @@
       </c>
     </row>
     <row r="235" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A235" s="9" t="s">
+      <c r="A235" s="8" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>